<commit_message>
Link budgets, pass charts, instrument view, Moon-of-date elements
- Link budgets (tools/linkbudget.py): station radio columns and a spacecraft
  Payloads sheet; live downlink/uplink Eb/N0 and margin in Show info
- Per-station charts (tools/charts.py): contact timeline, elevation and
  margin per pass, shown in a movable chart panel in the viewer
- Instrument view: camera nodes read from models/source/probe.glb
  (tools/instruments.py), full-screen sensor view with FOV frame
- Lunar elements in the Moon's equator of date
- Orbit lines, grid and links blended so they cast no shadows
- Movable, smaller panels; Earth and Moon grids
- groundstations.ods added (live station file)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/groundstations.xlsx
+++ b/groundstations.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -447,6 +447,9 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -495,6 +498,21 @@
           <t>Body</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Antenna gain (dBi)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>System noise temp (K)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Tx power (W)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -522,6 +540,15 @@
           <t>2-way</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v>35</v>
+      </c>
+      <c r="K2" t="n">
+        <v>150</v>
+      </c>
+      <c r="L2" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -554,9 +581,18 @@
           <t>Moon</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>20</v>
+      </c>
+      <c r="K3" t="n">
+        <v>250</v>
+      </c>
+      <c r="L3" t="n">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="12">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Name" prompt="Shown as the label in the viewer. Must be unique."/>
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Latitude" prompt="Decimal degrees, north positive (28.6083), or 28.6083 N, or 28 36 30.2 N."/>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Longitude" prompt="Decimal degrees, east positive (-80.6043), or 80.6043 W, or 80 36 15.6 W."/>
@@ -570,6 +606,9 @@
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Body" error="Choose Earth or Moon." promptTitle="Body" prompt="Earth or Moon. Blank = Earth. Moon: ground elevation is metres above the mean lunar radius (1737.4 km), blank = 0; it is not looked up." type="list">
       <formula1>"Earth,Moon"</formula1>
     </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Antenna gain" prompt="The station antenna's gain, dBi (e.g. a 3.7 m S-band dish ~37 dBi). Needed for link budgets."/>
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="System noise temperature" prompt="Receive system noise temperature, kelvin (e.g. 150 K). With the gain it gives the station's G/T."/>
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Transmit power" prompt="Uplink transmit power, watts. Only used for 2-way links."/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -581,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -718,7 +757,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -737,6 +775,30 @@
       <c r="A25" t="inlineStr">
         <is>
           <t>A station's link line and passes also need the line of sight to miss the Earth and the Moon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Antenna gain (dBi), System noise temp (K), Tx power (W) - columns J-L, optional: the station's radio for</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    link budgets. Gain and noise temperature give its G/T (downlink); Tx power its uplink (2-way only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    The spacecraft side is in spacecraft.xlsx, sheet Payloads. The example values are illustrative.</t>
         </is>
       </c>
     </row>

</xml_diff>